<commit_message>
feat: refine import export problems and escalation
</commit_message>
<xml_diff>
--- a/templates/Template_Escalonamento.xlsx
+++ b/templates/Template_Escalonamento.xlsx
@@ -401,41 +401,41 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AI15"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="12.83203125" customWidth="1"/>
-    <col min="14" max="14" width="12.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
-    <col min="16" max="16" width="12.83203125" customWidth="1"/>
-    <col min="17" max="17" width="12.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" customWidth="1"/>
-    <col min="19" max="19" width="12.83203125" customWidth="1"/>
-    <col min="20" max="20" width="12.83203125" customWidth="1"/>
-    <col min="21" max="21" width="12.83203125" customWidth="1"/>
-    <col min="22" max="22" width="12.83203125" customWidth="1"/>
-    <col min="23" max="23" width="12.83203125" customWidth="1"/>
-    <col min="24" max="24" width="12.83203125" customWidth="1"/>
-    <col min="25" max="25" width="12.83203125" customWidth="1"/>
-    <col min="26" max="26" width="12.83203125" customWidth="1"/>
-    <col min="27" max="27" width="12.83203125" customWidth="1"/>
-    <col min="28" max="28" width="12.83203125" customWidth="1"/>
-    <col min="29" max="29" width="12.83203125" customWidth="1"/>
-    <col min="30" max="30" width="12.83203125" customWidth="1"/>
-    <col min="31" max="31" width="12.83203125" customWidth="1"/>
-    <col min="32" max="32" width="12.83203125" customWidth="1"/>
-    <col min="33" max="33" width="12.83203125" customWidth="1"/>
-    <col min="34" max="34" width="12.83203125" customWidth="1"/>
-    <col min="35" max="35" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="13.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="8" max="8" width="13.83203125" customWidth="1"/>
+    <col min="9" max="9" width="13.83203125" customWidth="1"/>
+    <col min="10" max="10" width="13.83203125" customWidth="1"/>
+    <col min="11" max="11" width="13.83203125" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="13" max="13" width="13.83203125" customWidth="1"/>
+    <col min="14" max="14" width="13.83203125" customWidth="1"/>
+    <col min="15" max="15" width="13.83203125" customWidth="1"/>
+    <col min="16" max="16" width="13.83203125" customWidth="1"/>
+    <col min="17" max="17" width="13.83203125" customWidth="1"/>
+    <col min="18" max="18" width="13.83203125" customWidth="1"/>
+    <col min="19" max="19" width="13.83203125" customWidth="1"/>
+    <col min="20" max="20" width="13.83203125" customWidth="1"/>
+    <col min="21" max="21" width="13.83203125" customWidth="1"/>
+    <col min="22" max="22" width="13.83203125" customWidth="1"/>
+    <col min="23" max="23" width="13.83203125" customWidth="1"/>
+    <col min="24" max="24" width="13.83203125" customWidth="1"/>
+    <col min="25" max="25" width="13.83203125" customWidth="1"/>
+    <col min="26" max="26" width="13.83203125" customWidth="1"/>
+    <col min="27" max="27" width="13.83203125" customWidth="1"/>
+    <col min="28" max="28" width="13.83203125" customWidth="1"/>
+    <col min="29" max="29" width="13.83203125" customWidth="1"/>
+    <col min="30" max="30" width="13.83203125" customWidth="1"/>
+    <col min="31" max="31" width="13.83203125" customWidth="1"/>
+    <col min="32" max="32" width="13.83203125" customWidth="1"/>
+    <col min="33" max="33" width="13.83203125" customWidth="1"/>
+    <col min="34" max="34" width="13.83203125" customWidth="1"/>
+    <col min="35" max="35" width="13.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -445,7 +445,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Julho/2026</v>
+        <v>Mês/Ano: (Selecione o mês correto direto no painel do sistema)</v>
       </c>
     </row>
     <row r="4">
@@ -1516,41 +1516,41 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:AI9"/>
   <cols>
-    <col min="1" max="1" width="32.83203125" customWidth="1"/>
-    <col min="2" max="2" width="22.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="12.83203125" customWidth="1"/>
-    <col min="5" max="5" width="12.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="12.83203125" customWidth="1"/>
-    <col min="9" max="9" width="12.83203125" customWidth="1"/>
-    <col min="10" max="10" width="12.83203125" customWidth="1"/>
-    <col min="11" max="11" width="12.83203125" customWidth="1"/>
-    <col min="12" max="12" width="12.83203125" customWidth="1"/>
-    <col min="13" max="13" width="12.83203125" customWidth="1"/>
-    <col min="14" max="14" width="12.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
-    <col min="16" max="16" width="12.83203125" customWidth="1"/>
-    <col min="17" max="17" width="12.83203125" customWidth="1"/>
-    <col min="18" max="18" width="12.83203125" customWidth="1"/>
-    <col min="19" max="19" width="12.83203125" customWidth="1"/>
-    <col min="20" max="20" width="12.83203125" customWidth="1"/>
-    <col min="21" max="21" width="12.83203125" customWidth="1"/>
-    <col min="22" max="22" width="12.83203125" customWidth="1"/>
-    <col min="23" max="23" width="12.83203125" customWidth="1"/>
-    <col min="24" max="24" width="12.83203125" customWidth="1"/>
-    <col min="25" max="25" width="12.83203125" customWidth="1"/>
-    <col min="26" max="26" width="12.83203125" customWidth="1"/>
-    <col min="27" max="27" width="12.83203125" customWidth="1"/>
-    <col min="28" max="28" width="12.83203125" customWidth="1"/>
-    <col min="29" max="29" width="12.83203125" customWidth="1"/>
-    <col min="30" max="30" width="12.83203125" customWidth="1"/>
-    <col min="31" max="31" width="12.83203125" customWidth="1"/>
-    <col min="32" max="32" width="12.83203125" customWidth="1"/>
-    <col min="33" max="33" width="12.83203125" customWidth="1"/>
-    <col min="34" max="34" width="12.83203125" customWidth="1"/>
-    <col min="35" max="35" width="12.83203125" customWidth="1"/>
+    <col min="1" max="1" width="35.83203125" customWidth="1"/>
+    <col min="2" max="2" width="25.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="15.83203125" customWidth="1"/>
+    <col min="5" max="5" width="13.83203125" customWidth="1"/>
+    <col min="6" max="6" width="13.83203125" customWidth="1"/>
+    <col min="7" max="7" width="13.83203125" customWidth="1"/>
+    <col min="8" max="8" width="13.83203125" customWidth="1"/>
+    <col min="9" max="9" width="13.83203125" customWidth="1"/>
+    <col min="10" max="10" width="13.83203125" customWidth="1"/>
+    <col min="11" max="11" width="13.83203125" customWidth="1"/>
+    <col min="12" max="12" width="13.83203125" customWidth="1"/>
+    <col min="13" max="13" width="13.83203125" customWidth="1"/>
+    <col min="14" max="14" width="13.83203125" customWidth="1"/>
+    <col min="15" max="15" width="13.83203125" customWidth="1"/>
+    <col min="16" max="16" width="13.83203125" customWidth="1"/>
+    <col min="17" max="17" width="13.83203125" customWidth="1"/>
+    <col min="18" max="18" width="13.83203125" customWidth="1"/>
+    <col min="19" max="19" width="13.83203125" customWidth="1"/>
+    <col min="20" max="20" width="13.83203125" customWidth="1"/>
+    <col min="21" max="21" width="13.83203125" customWidth="1"/>
+    <col min="22" max="22" width="13.83203125" customWidth="1"/>
+    <col min="23" max="23" width="13.83203125" customWidth="1"/>
+    <col min="24" max="24" width="13.83203125" customWidth="1"/>
+    <col min="25" max="25" width="13.83203125" customWidth="1"/>
+    <col min="26" max="26" width="13.83203125" customWidth="1"/>
+    <col min="27" max="27" width="13.83203125" customWidth="1"/>
+    <col min="28" max="28" width="13.83203125" customWidth="1"/>
+    <col min="29" max="29" width="13.83203125" customWidth="1"/>
+    <col min="30" max="30" width="13.83203125" customWidth="1"/>
+    <col min="31" max="31" width="13.83203125" customWidth="1"/>
+    <col min="32" max="32" width="13.83203125" customWidth="1"/>
+    <col min="33" max="33" width="13.83203125" customWidth="1"/>
+    <col min="34" max="34" width="13.83203125" customWidth="1"/>
+    <col min="35" max="35" width="13.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1560,7 +1560,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Mês/Ano (ex: Agosto/2026)</v>
+        <v>Mês/Ano: (Selecione o mês correto direto no painel do sistema antes de importar)</v>
       </c>
     </row>
     <row r="4">
@@ -2214,7 +2214,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A45"/>
+  <dimension ref="A1:A34"/>
   <cols>
     <col min="1" max="1" width="90.83203125" customWidth="1"/>
   </cols>
@@ -2236,7 +2236,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>• O nome da aba identifica a área (ex: "DevOps - Cloud", "PDV", "Redes")</v>
+        <v>• O nome da aba identifica a área no sistema (ex: "DevOps", "PDV", "Redes")</v>
       </c>
     </row>
     <row r="7">
@@ -2246,17 +2246,17 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>• Linha 1: Nome da área (será usado para identificar no sistema)</v>
+        <v>• Linha 1: Nome da área (importante para identificação)</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>• Linha 2: Mês/Ano de referência (ex: "Julho/2026", "Agosto/2026")</v>
+        <v>• Linha 2: Informativa (O Mês e Ano reais agora são selecionados na tela do sistema antes de importar!)</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>• Linha 3: Vazia (separador)</v>
+        <v>• Linha 3: Vazia (apenas para separação visual)</v>
       </c>
     </row>
     <row r="11">
@@ -2301,117 +2301,67 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>• Preencher com o horário do sobreaviso naquele dia</v>
+        <v>• Preencha com o horário do sobreaviso naquele dia</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>• Formatos aceitos:</v>
+        <v>• Formatos recomendados:</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v xml:space="preserve">    - "18:00-06:00" (horário início - horário fim)</v>
+        <v xml:space="preserve">    - "18:00-06:00" (horário de início e fim separados por hífen)</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v xml:space="preserve">    - "18:00 às 06:00" (com "às")</v>
+        <v xml:space="preserve">    - "24hs" ou "X" (para sinalizar um plantão de dia inteiro)</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v xml:space="preserve">    - "08:00-08:00" (turno de 24h)</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v xml:space="preserve">    - "24hs" ou "24h" (turno integral)</v>
+        <v xml:space="preserve">    - Deixe VAZIO se não houver plantão no dia</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v xml:space="preserve">    - "X" ou "S" (marca presença como 24h)</v>
+        <v>DICAS E REGRAS DA IMPORTAÇÃO:</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v xml:space="preserve">    - Vazio = sem plantão nesse dia</v>
+        <v>• SELECIONE O MÊS/ANO NO SISTEMA: A planilha será importada para o mês que você selecionar na tela de Importação.</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>• A importação substitui toda a escala do mês selecionado para aquela área.</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>REGRAS DE IMPORTAÇÃO:</v>
+        <v>• Plantonistas novos que não existiam no sistema serão criados automaticamente.</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>• A importação SUBSTITUI toda a escala do mês para a área</v>
+        <v>• Não proteja a planilha com senha, senão o sistema não conseguirá ler os dados.</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>• Plantonistas novos são criados automaticamente (senha padrão: plantonista123)</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>• Plantonistas existentes são atualizados (cargo, contato)</v>
+        <v>• Múltiplas áreas podem ser importadas juntas, basta criar várias abas no mesmo arquivo Excel.</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>• Conflitos são detectados (mesmo plantonista em dois turnos sobrepostos)</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="str">
-        <v>• Níveis 2º, 3º, 4º não precisam ter dias preenchidos (são escalação fixa)</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="str">
-        <v>MÚLTIPLAS ÁREAS:</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="str">
-        <v>• Crie uma aba para cada área no mesmo arquivo</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="str">
-        <v>• Ou envie arquivos separados por área</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="str">
-        <v>DICAS:</v>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="str">
-        <v>• Não use proteção por senha no arquivo</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="str">
-        <v>• Aceita formatos .xlsx e .csv</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="str">
-        <v>• O sistema valida os dados antes de importar</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="str">
-        <v>• Veja a aba "DevOps - Cloud" como exemplo preenchido</v>
+        <v>👉 Veja a aba "DevOps - Cloud" neste arquivo como um exemplo prático já preenchido!</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A45"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A34"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>